<commit_message>
Web3 Payment Gateway and PDF Reporting System
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -37,7 +37,7 @@
     <t>PH-001</t>
   </si>
   <si>
-    <t>خلاص</t>
+    <t>Saleh</t>
   </si>
   <si>
     <t>عالي</t>
@@ -49,7 +49,7 @@
     <t>PH-002</t>
   </si>
   <si>
-    <t>سكري</t>
+    <t>Sukkar</t>
   </si>
   <si>
     <t>متوسط</t>
@@ -111,10 +111,10 @@
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
+    <xf borderId="0" fillId="0" fontId="1" numFmtId="9" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+      <alignment readingOrder="0"/>
+    </xf>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="9" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="3" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
@@ -369,19 +369,19 @@
       <c r="A2" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="2" t="s">
         <v>8</v>
       </c>
       <c r="C2" s="2">
         <v>180.0</v>
       </c>
-      <c r="D2" s="4">
+      <c r="D2" s="3">
         <v>0.12</v>
       </c>
-      <c r="E2" s="3" t="s">
+      <c r="E2" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="F2" s="3" t="s">
+      <c r="F2" s="4" t="s">
         <v>10</v>
       </c>
     </row>
@@ -389,19 +389,19 @@
       <c r="A3" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="B3" s="2" t="s">
         <v>12</v>
       </c>
       <c r="C3" s="2">
         <v>210.0</v>
       </c>
-      <c r="D3" s="4">
+      <c r="D3" s="3">
         <v>0.15</v>
       </c>
-      <c r="E3" s="3" t="s">
+      <c r="E3" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="F3" s="3" t="s">
+      <c r="F3" s="4" t="s">
         <v>14</v>
       </c>
     </row>

</xml_diff>